<commit_message>
Update CVP/SWP allocation percentages through 2025
</commit_message>
<xml_diff>
--- a/raw/cvp/allocations.xlsx
+++ b/raw/cvp/allocations.xlsx
@@ -1,25 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24729"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffh\OneDrive\Documents\UCDavis\data-surface-water\raw\cvp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\data-surface-water\raw\cvp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE45F8F-D8E3-4EF2-8B45-384885B623FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4BE5148-2185-484D-9C29-6DC85EDC6BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="7965" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="allocations" sheetId="1" r:id="rId1"/>
     <sheet name="lookup" sheetId="5" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -532,209 +543,220 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AT15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="A1:AX15"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="42" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="4.68359375" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="8.83984375" customWidth="1"/>
+    <col min="2" max="10" width="9.23046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:50" x14ac:dyDescent="0.4">
       <c r="B1">
+        <v>2025</v>
+      </c>
+      <c r="C1">
+        <v>2024</v>
+      </c>
+      <c r="D1">
+        <v>2023</v>
+      </c>
+      <c r="E1">
+        <v>2022</v>
+      </c>
+      <c r="F1">
         <v>2021</v>
       </c>
-      <c r="C1">
+      <c r="G1">
         <v>2020</v>
       </c>
-      <c r="D1">
+      <c r="H1">
         <v>2019</v>
       </c>
-      <c r="E1">
+      <c r="I1">
         <v>2018</v>
       </c>
-      <c r="F1">
+      <c r="J1">
         <v>2017</v>
       </c>
-      <c r="G1">
+      <c r="K1">
         <v>2016</v>
       </c>
-      <c r="H1">
+      <c r="L1">
         <v>2015</v>
       </c>
-      <c r="I1">
+      <c r="M1">
         <v>2014</v>
       </c>
-      <c r="J1">
+      <c r="N1">
         <v>2013</v>
       </c>
-      <c r="K1">
+      <c r="O1">
         <v>2012</v>
       </c>
-      <c r="L1">
+      <c r="P1">
         <v>2011</v>
       </c>
-      <c r="M1">
+      <c r="Q1">
         <v>2010</v>
       </c>
-      <c r="N1">
+      <c r="R1">
         <v>2009</v>
       </c>
-      <c r="O1">
+      <c r="S1">
         <v>2008</v>
       </c>
-      <c r="P1">
+      <c r="T1">
         <v>2007</v>
       </c>
-      <c r="Q1">
+      <c r="U1">
         <v>2006</v>
       </c>
-      <c r="R1">
+      <c r="V1">
         <v>2005</v>
       </c>
-      <c r="S1">
+      <c r="W1">
         <v>2004</v>
       </c>
-      <c r="T1">
+      <c r="X1">
         <v>2003</v>
       </c>
-      <c r="U1">
+      <c r="Y1">
         <v>2002</v>
       </c>
-      <c r="V1">
+      <c r="Z1">
         <v>2001</v>
       </c>
-      <c r="W1">
+      <c r="AA1">
         <v>2000</v>
       </c>
-      <c r="X1">
+      <c r="AB1">
         <v>1999</v>
       </c>
-      <c r="Y1">
+      <c r="AC1">
         <v>1998</v>
       </c>
-      <c r="Z1">
+      <c r="AD1">
         <v>1997</v>
       </c>
-      <c r="AA1">
+      <c r="AE1">
         <v>1996</v>
       </c>
-      <c r="AB1">
+      <c r="AF1">
         <v>1995</v>
       </c>
-      <c r="AC1">
+      <c r="AG1">
         <v>1994</v>
       </c>
-      <c r="AD1">
+      <c r="AH1">
         <v>1993</v>
       </c>
-      <c r="AE1">
+      <c r="AI1">
         <v>1992</v>
       </c>
-      <c r="AF1">
+      <c r="AJ1">
         <v>1991</v>
       </c>
-      <c r="AG1">
+      <c r="AK1">
         <v>1990</v>
       </c>
-      <c r="AH1">
+      <c r="AL1">
         <v>1989</v>
       </c>
-      <c r="AI1">
+      <c r="AM1">
         <v>1988</v>
       </c>
-      <c r="AJ1">
+      <c r="AN1">
         <v>1987</v>
       </c>
-      <c r="AK1">
+      <c r="AO1">
         <v>1986</v>
       </c>
-      <c r="AL1">
+      <c r="AP1">
         <v>1985</v>
       </c>
-      <c r="AM1">
+      <c r="AQ1">
         <v>1984</v>
       </c>
-      <c r="AN1">
+      <c r="AR1">
         <v>1983</v>
       </c>
-      <c r="AO1">
+      <c r="AS1">
         <v>1982</v>
       </c>
-      <c r="AP1">
+      <c r="AT1">
         <v>1981</v>
       </c>
-      <c r="AQ1">
+      <c r="AU1">
         <v>1980</v>
       </c>
-      <c r="AR1">
+      <c r="AV1">
         <v>1979</v>
       </c>
-      <c r="AS1">
+      <c r="AW1">
         <v>1978</v>
       </c>
-      <c r="AT1">
+      <c r="AX1">
         <v>1977</v>
       </c>
     </row>
-    <row r="2" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C2">
+        <v>100</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
         <v>50</v>
       </c>
-      <c r="D2">
-        <v>100</v>
-      </c>
-      <c r="E2">
-        <v>100</v>
-      </c>
-      <c r="F2">
-        <v>100</v>
-      </c>
-      <c r="G2">
-        <v>100</v>
-      </c>
       <c r="H2">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J2">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="K2">
         <v>100</v>
       </c>
       <c r="L2">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="N2">
+        <v>75</v>
+      </c>
+      <c r="O2">
+        <v>100</v>
+      </c>
+      <c r="P2">
+        <v>100</v>
+      </c>
+      <c r="Q2">
+        <v>100</v>
+      </c>
+      <c r="R2">
         <v>40</v>
       </c>
-      <c r="O2">
+      <c r="S2">
         <v>40</v>
       </c>
-      <c r="P2">
-        <v>100</v>
-      </c>
-      <c r="Q2">
-        <v>100</v>
-      </c>
-      <c r="R2">
-        <v>100</v>
-      </c>
-      <c r="S2">
-        <v>100</v>
-      </c>
       <c r="T2">
         <v>100</v>
       </c>
@@ -742,53 +764,53 @@
         <v>100</v>
       </c>
       <c r="V2">
+        <v>100</v>
+      </c>
+      <c r="W2">
+        <v>100</v>
+      </c>
+      <c r="X2">
+        <v>100</v>
+      </c>
+      <c r="Y2">
+        <v>100</v>
+      </c>
+      <c r="Z2">
         <v>60</v>
       </c>
-      <c r="W2">
-        <v>100</v>
-      </c>
-      <c r="X2">
-        <v>100</v>
-      </c>
-      <c r="Y2">
-        <v>100</v>
-      </c>
-      <c r="Z2">
+      <c r="AA2">
+        <v>100</v>
+      </c>
+      <c r="AB2">
+        <v>100</v>
+      </c>
+      <c r="AC2">
+        <v>100</v>
+      </c>
+      <c r="AD2">
         <v>90</v>
       </c>
-      <c r="AA2">
-        <v>100</v>
-      </c>
-      <c r="AB2">
-        <v>100</v>
-      </c>
-      <c r="AC2">
+      <c r="AE2">
+        <v>100</v>
+      </c>
+      <c r="AF2">
+        <v>100</v>
+      </c>
+      <c r="AG2">
         <v>35</v>
       </c>
-      <c r="AD2">
-        <v>100</v>
-      </c>
-      <c r="AE2">
+      <c r="AH2">
+        <v>100</v>
+      </c>
+      <c r="AI2">
         <v>25</v>
       </c>
-      <c r="AF2">
+      <c r="AJ2">
         <v>25</v>
       </c>
-      <c r="AG2">
+      <c r="AK2">
         <v>50</v>
       </c>
-      <c r="AH2">
-        <v>100</v>
-      </c>
-      <c r="AI2">
-        <v>100</v>
-      </c>
-      <c r="AJ2">
-        <v>100</v>
-      </c>
-      <c r="AK2">
-        <v>100</v>
-      </c>
       <c r="AL2">
         <v>100</v>
       </c>
@@ -814,54 +836,66 @@
         <v>100</v>
       </c>
       <c r="AT2">
+        <v>100</v>
+      </c>
+      <c r="AU2">
+        <v>100</v>
+      </c>
+      <c r="AV2">
+        <v>100</v>
+      </c>
+      <c r="AW2">
+        <v>100</v>
+      </c>
+      <c r="AX2">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3">
+        <v>100</v>
+      </c>
+      <c r="C3">
+        <v>100</v>
+      </c>
+      <c r="D3">
+        <v>100</v>
+      </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3">
         <v>25</v>
       </c>
-      <c r="C3">
-        <v>75</v>
-      </c>
-      <c r="D3">
-        <v>100</v>
-      </c>
-      <c r="E3">
-        <v>100</v>
-      </c>
-      <c r="F3">
-        <v>100</v>
-      </c>
       <c r="G3">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="H3">
+        <v>100</v>
+      </c>
+      <c r="I3">
+        <v>100</v>
+      </c>
+      <c r="J3">
+        <v>100</v>
+      </c>
+      <c r="K3">
+        <v>100</v>
+      </c>
+      <c r="L3">
         <v>25</v>
       </c>
-      <c r="I3">
+      <c r="M3">
         <v>50</v>
       </c>
-      <c r="J3">
-        <v>100</v>
-      </c>
-      <c r="K3">
-        <v>100</v>
-      </c>
-      <c r="L3">
-        <v>100</v>
-      </c>
-      <c r="M3">
-        <v>100</v>
-      </c>
       <c r="N3">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="O3">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="P3">
         <v>100</v>
@@ -870,10 +904,10 @@
         <v>100</v>
       </c>
       <c r="R3">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="S3">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="T3">
         <v>100</v>
@@ -882,19 +916,19 @@
         <v>100</v>
       </c>
       <c r="V3">
+        <v>100</v>
+      </c>
+      <c r="W3">
+        <v>100</v>
+      </c>
+      <c r="X3">
+        <v>100</v>
+      </c>
+      <c r="Y3">
+        <v>100</v>
+      </c>
+      <c r="Z3">
         <v>85</v>
-      </c>
-      <c r="W3">
-        <v>100</v>
-      </c>
-      <c r="X3">
-        <v>95</v>
-      </c>
-      <c r="Y3">
-        <v>100</v>
-      </c>
-      <c r="Z3">
-        <v>95</v>
       </c>
       <c r="AA3">
         <v>100</v>
@@ -903,32 +937,32 @@
         <v>95</v>
       </c>
       <c r="AC3">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AD3">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="AE3">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AF3">
+        <v>95</v>
+      </c>
+      <c r="AG3">
+        <v>75</v>
+      </c>
+      <c r="AH3">
+        <v>100</v>
+      </c>
+      <c r="AI3">
+        <v>75</v>
+      </c>
+      <c r="AJ3">
         <v>37.5</v>
       </c>
-      <c r="AG3">
+      <c r="AK3">
         <v>62.5</v>
       </c>
-      <c r="AH3">
-        <v>100</v>
-      </c>
-      <c r="AI3">
-        <v>100</v>
-      </c>
-      <c r="AJ3">
-        <v>100</v>
-      </c>
-      <c r="AK3">
-        <v>100</v>
-      </c>
       <c r="AL3">
         <v>100</v>
       </c>
@@ -954,15 +988,27 @@
         <v>100</v>
       </c>
       <c r="AT3">
+        <v>100</v>
+      </c>
+      <c r="AU3">
+        <v>100</v>
+      </c>
+      <c r="AV3">
+        <v>100</v>
+      </c>
+      <c r="AW3">
+        <v>100</v>
+      </c>
+      <c r="AX3">
         <v>37.5</v>
       </c>
     </row>
-    <row r="4" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C4">
         <v>100</v>
@@ -971,19 +1017,19 @@
         <v>100</v>
       </c>
       <c r="E4">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="F4">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G4">
         <v>100</v>
       </c>
       <c r="H4">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="I4">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="J4">
         <v>100</v>
@@ -992,10 +1038,10 @@
         <v>100</v>
       </c>
       <c r="L4">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="M4">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="N4">
         <v>100</v>
@@ -1043,21 +1089,33 @@
         <v>100</v>
       </c>
       <c r="AC4">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AD4">
         <v>100</v>
       </c>
       <c r="AE4">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+        <v>100</v>
+      </c>
+      <c r="AF4">
+        <v>100</v>
+      </c>
+      <c r="AG4">
+        <v>75</v>
+      </c>
+      <c r="AH4">
+        <v>100</v>
+      </c>
+      <c r="AI4">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -1066,19 +1124,19 @@
         <v>100</v>
       </c>
       <c r="E5">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="F5">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G5">
         <v>100</v>
       </c>
       <c r="H5">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="I5">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="J5">
         <v>100</v>
@@ -1087,10 +1145,10 @@
         <v>100</v>
       </c>
       <c r="L5">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="M5">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="N5">
         <v>100</v>
@@ -1138,28 +1196,28 @@
         <v>100</v>
       </c>
       <c r="AC5">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AD5">
         <v>100</v>
       </c>
       <c r="AE5">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AF5">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AG5">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AH5">
         <v>100</v>
       </c>
       <c r="AI5">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AJ5">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AK5">
         <v>100</v>
@@ -1189,197 +1247,233 @@
         <v>100</v>
       </c>
       <c r="AT5">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+        <v>100</v>
+      </c>
+      <c r="AU5">
+        <v>100</v>
+      </c>
+      <c r="AV5">
+        <v>100</v>
+      </c>
+      <c r="AW5">
+        <v>100</v>
+      </c>
+      <c r="AX5">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="C6">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D6">
         <v>100</v>
       </c>
       <c r="E6">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F6">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G6">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="H6">
+        <v>100</v>
+      </c>
+      <c r="I6">
+        <v>100</v>
+      </c>
+      <c r="J6">
+        <v>100</v>
+      </c>
+      <c r="K6">
+        <v>100</v>
+      </c>
+      <c r="L6">
         <v>25</v>
       </c>
-      <c r="I6">
+      <c r="M6">
         <v>50</v>
       </c>
-      <c r="J6">
-        <v>75</v>
-      </c>
-      <c r="K6">
-        <v>100</v>
-      </c>
-      <c r="L6">
-        <v>100</v>
-      </c>
-      <c r="M6">
-        <v>100</v>
-      </c>
       <c r="N6">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+        <v>75</v>
+      </c>
+      <c r="O6">
+        <v>100</v>
+      </c>
+      <c r="P6">
+        <v>100</v>
+      </c>
+      <c r="Q6">
+        <v>100</v>
+      </c>
+      <c r="R6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>4</v>
       </c>
       <c r="B7">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="C7">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D7">
         <v>100</v>
       </c>
       <c r="E7">
-        <v>100</v>
+        <v>33</v>
       </c>
       <c r="F7">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G7">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="H7">
+        <v>100</v>
+      </c>
+      <c r="I7">
+        <v>100</v>
+      </c>
+      <c r="J7">
+        <v>100</v>
+      </c>
+      <c r="K7">
+        <v>100</v>
+      </c>
+      <c r="L7">
         <v>25</v>
       </c>
-      <c r="I7">
+      <c r="M7">
         <v>50</v>
       </c>
-      <c r="J7">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+      <c r="N7">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>5</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="C8">
+        <v>50</v>
+      </c>
+      <c r="D8">
+        <v>100</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
         <v>20</v>
       </c>
-      <c r="D8">
-        <v>75</v>
-      </c>
-      <c r="E8">
+      <c r="H8">
+        <v>75</v>
+      </c>
+      <c r="I8">
         <v>50</v>
       </c>
-      <c r="F8">
-        <v>100</v>
-      </c>
-      <c r="G8">
+      <c r="J8">
+        <v>100</v>
+      </c>
+      <c r="K8">
         <v>5</v>
       </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
         <v>20</v>
-      </c>
-      <c r="K8">
-        <v>40</v>
-      </c>
-      <c r="L8">
-        <v>80</v>
-      </c>
-      <c r="M8">
-        <v>45</v>
-      </c>
-      <c r="N8">
-        <v>10</v>
       </c>
       <c r="O8">
         <v>40</v>
       </c>
       <c r="P8">
+        <v>80</v>
+      </c>
+      <c r="Q8">
+        <v>45</v>
+      </c>
+      <c r="R8">
+        <v>10</v>
+      </c>
+      <c r="S8">
+        <v>40</v>
+      </c>
+      <c r="T8">
         <v>50</v>
       </c>
-      <c r="Q8">
-        <v>100</v>
-      </c>
-      <c r="R8">
+      <c r="U8">
+        <v>100</v>
+      </c>
+      <c r="V8">
         <v>85</v>
       </c>
-      <c r="S8">
+      <c r="W8">
         <v>70</v>
       </c>
-      <c r="T8">
-        <v>75</v>
-      </c>
-      <c r="U8">
+      <c r="X8">
+        <v>75</v>
+      </c>
+      <c r="Y8">
         <v>70</v>
       </c>
-      <c r="V8">
+      <c r="Z8">
         <v>49</v>
       </c>
-      <c r="W8">
+      <c r="AA8">
         <v>65</v>
       </c>
-      <c r="X8">
+      <c r="AB8">
         <v>70</v>
       </c>
-      <c r="Y8">
-        <v>100</v>
-      </c>
-      <c r="Z8">
+      <c r="AC8">
+        <v>100</v>
+      </c>
+      <c r="AD8">
         <v>90</v>
       </c>
-      <c r="AA8">
+      <c r="AE8">
         <v>95</v>
       </c>
-      <c r="AB8">
-        <v>100</v>
-      </c>
-      <c r="AC8">
+      <c r="AF8">
+        <v>100</v>
+      </c>
+      <c r="AG8">
         <v>35</v>
       </c>
-      <c r="AD8">
+      <c r="AH8">
         <v>50</v>
       </c>
-      <c r="AE8">
+      <c r="AI8">
         <v>25</v>
       </c>
-      <c r="AF8">
+      <c r="AJ8">
         <v>25</v>
       </c>
-      <c r="AG8">
+      <c r="AK8">
         <v>50</v>
       </c>
-      <c r="AH8">
-        <v>100</v>
-      </c>
-      <c r="AI8">
-        <v>100</v>
-      </c>
-      <c r="AJ8">
-        <v>100</v>
-      </c>
-      <c r="AK8">
-        <v>100</v>
-      </c>
       <c r="AL8">
         <v>100</v>
       </c>
@@ -1405,121 +1499,133 @@
         <v>100</v>
       </c>
       <c r="AT8">
+        <v>100</v>
+      </c>
+      <c r="AU8">
+        <v>100</v>
+      </c>
+      <c r="AV8">
+        <v>100</v>
+      </c>
+      <c r="AW8">
+        <v>100</v>
+      </c>
+      <c r="AX8">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9">
+        <v>80</v>
+      </c>
+      <c r="C9">
+        <v>75</v>
+      </c>
+      <c r="D9">
+        <v>100</v>
+      </c>
+      <c r="E9">
+        <v>33</v>
+      </c>
+      <c r="F9">
         <v>25</v>
       </c>
-      <c r="C9">
+      <c r="G9">
         <v>70</v>
       </c>
-      <c r="D9">
-        <v>100</v>
-      </c>
-      <c r="E9">
-        <v>75</v>
-      </c>
-      <c r="F9">
-        <v>100</v>
-      </c>
-      <c r="G9">
+      <c r="H9">
+        <v>100</v>
+      </c>
+      <c r="I9">
+        <v>75</v>
+      </c>
+      <c r="J9">
+        <v>100</v>
+      </c>
+      <c r="K9">
         <v>55</v>
       </c>
-      <c r="H9">
+      <c r="L9">
         <v>25</v>
       </c>
-      <c r="I9">
+      <c r="M9">
         <v>50</v>
       </c>
-      <c r="J9">
+      <c r="N9">
         <v>70</v>
       </c>
-      <c r="K9">
-        <v>75</v>
-      </c>
-      <c r="L9">
-        <v>100</v>
-      </c>
-      <c r="M9">
-        <v>75</v>
-      </c>
-      <c r="N9">
+      <c r="O9">
+        <v>75</v>
+      </c>
+      <c r="P9">
+        <v>100</v>
+      </c>
+      <c r="Q9">
+        <v>75</v>
+      </c>
+      <c r="R9">
         <v>60</v>
       </c>
-      <c r="O9">
-        <v>75</v>
-      </c>
-      <c r="P9">
-        <v>75</v>
-      </c>
-      <c r="Q9">
-        <v>100</v>
-      </c>
-      <c r="R9">
-        <v>100</v>
-      </c>
       <c r="S9">
+        <v>75</v>
+      </c>
+      <c r="T9">
+        <v>75</v>
+      </c>
+      <c r="U9">
+        <v>100</v>
+      </c>
+      <c r="V9">
+        <v>100</v>
+      </c>
+      <c r="W9">
         <v>95</v>
       </c>
-      <c r="T9">
-        <v>100</v>
-      </c>
-      <c r="U9">
+      <c r="X9">
+        <v>100</v>
+      </c>
+      <c r="Y9">
         <v>95</v>
       </c>
-      <c r="V9">
+      <c r="Z9">
         <v>77</v>
       </c>
-      <c r="W9">
+      <c r="AA9">
         <v>90</v>
       </c>
-      <c r="X9">
+      <c r="AB9">
         <v>95</v>
       </c>
-      <c r="Y9">
-        <v>100</v>
-      </c>
-      <c r="Z9">
+      <c r="AC9">
+        <v>100</v>
+      </c>
+      <c r="AD9">
         <v>95</v>
       </c>
-      <c r="AA9">
-        <v>100</v>
-      </c>
-      <c r="AB9">
-        <v>100</v>
-      </c>
-      <c r="AC9">
-        <v>75</v>
-      </c>
-      <c r="AD9">
-        <v>75</v>
-      </c>
       <c r="AE9">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AF9">
+        <v>100</v>
+      </c>
+      <c r="AG9">
+        <v>75</v>
+      </c>
+      <c r="AH9">
+        <v>75</v>
+      </c>
+      <c r="AI9">
+        <v>75</v>
+      </c>
+      <c r="AJ9">
         <v>37.5</v>
       </c>
-      <c r="AG9">
+      <c r="AK9">
         <v>62.5</v>
       </c>
-      <c r="AH9">
-        <v>100</v>
-      </c>
-      <c r="AI9">
-        <v>100</v>
-      </c>
-      <c r="AJ9">
-        <v>100</v>
-      </c>
-      <c r="AK9">
-        <v>100</v>
-      </c>
       <c r="AL9">
         <v>100</v>
       </c>
@@ -1545,15 +1651,27 @@
         <v>100</v>
       </c>
       <c r="AT9">
+        <v>100</v>
+      </c>
+      <c r="AU9">
+        <v>100</v>
+      </c>
+      <c r="AV9">
+        <v>100</v>
+      </c>
+      <c r="AW9">
+        <v>100</v>
+      </c>
+      <c r="AX9">
         <v>37.5</v>
       </c>
     </row>
-    <row r="10" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>7</v>
       </c>
       <c r="B10">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C10">
         <v>100</v>
@@ -1562,32 +1680,32 @@
         <v>100</v>
       </c>
       <c r="E10">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F10">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G10">
         <v>100</v>
       </c>
       <c r="H10">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="I10">
+        <v>100</v>
+      </c>
+      <c r="J10">
+        <v>100</v>
+      </c>
+      <c r="K10">
+        <v>100</v>
+      </c>
+      <c r="L10">
+        <v>75</v>
+      </c>
+      <c r="M10">
         <v>65</v>
       </c>
-      <c r="J10">
-        <v>100</v>
-      </c>
-      <c r="K10">
-        <v>100</v>
-      </c>
-      <c r="L10">
-        <v>100</v>
-      </c>
-      <c r="M10">
-        <v>100</v>
-      </c>
       <c r="N10">
         <v>100</v>
       </c>
@@ -1634,21 +1752,33 @@
         <v>100</v>
       </c>
       <c r="AC10">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AD10">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AE10">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="11" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+        <v>100</v>
+      </c>
+      <c r="AF10">
+        <v>100</v>
+      </c>
+      <c r="AG10">
+        <v>75</v>
+      </c>
+      <c r="AH10">
+        <v>75</v>
+      </c>
+      <c r="AI10">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>8</v>
       </c>
       <c r="B11">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C11">
         <v>100</v>
@@ -1657,32 +1787,32 @@
         <v>100</v>
       </c>
       <c r="E11">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F11">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G11">
         <v>100</v>
       </c>
       <c r="H11">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="I11">
+        <v>100</v>
+      </c>
+      <c r="J11">
+        <v>100</v>
+      </c>
+      <c r="K11">
+        <v>100</v>
+      </c>
+      <c r="L11">
+        <v>75</v>
+      </c>
+      <c r="M11">
         <v>65</v>
       </c>
-      <c r="J11">
-        <v>100</v>
-      </c>
-      <c r="K11">
-        <v>100</v>
-      </c>
-      <c r="L11">
-        <v>100</v>
-      </c>
-      <c r="M11">
-        <v>100</v>
-      </c>
       <c r="N11">
         <v>100</v>
       </c>
@@ -1729,28 +1859,28 @@
         <v>100</v>
       </c>
       <c r="AC11">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AD11">
         <v>100</v>
       </c>
       <c r="AE11">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AF11">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="AG11">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AH11">
         <v>100</v>
       </c>
       <c r="AI11">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AJ11">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AK11">
         <v>100</v>
@@ -1780,16 +1910,25 @@
         <v>100</v>
       </c>
       <c r="AT11">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="12" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+        <v>100</v>
+      </c>
+      <c r="AU11">
+        <v>100</v>
+      </c>
+      <c r="AV11">
+        <v>100</v>
+      </c>
+      <c r="AW11">
+        <v>100</v>
+      </c>
+      <c r="AX11">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12">
-        <v>100</v>
-      </c>
       <c r="C12">
         <v>100</v>
       </c>
@@ -1797,133 +1936,145 @@
         <v>100</v>
       </c>
       <c r="E12">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F12">
         <v>100</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I12">
+        <v>100</v>
+      </c>
+      <c r="J12">
+        <v>100</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
         <v>85250</v>
       </c>
-      <c r="J12">
+      <c r="N12">
         <v>155000</v>
       </c>
-      <c r="K12">
+      <c r="O12">
         <v>155000</v>
       </c>
-      <c r="L12">
+      <c r="P12">
         <v>155000</v>
-      </c>
-      <c r="M12">
-        <v>155000</v>
-      </c>
-      <c r="N12">
-        <v>18000</v>
-      </c>
-      <c r="O12">
-        <v>35000</v>
-      </c>
-      <c r="P12">
-        <v>45000</v>
       </c>
       <c r="Q12">
         <v>155000</v>
       </c>
       <c r="R12">
+        <v>18000</v>
+      </c>
+      <c r="S12">
+        <v>35000</v>
+      </c>
+      <c r="T12">
+        <v>45000</v>
+      </c>
+      <c r="U12">
+        <v>155000</v>
+      </c>
+      <c r="V12">
         <v>43000</v>
       </c>
-      <c r="S12">
-        <v>0</v>
-      </c>
-      <c r="T12">
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
         <v>6</v>
       </c>
-      <c r="U12">
+      <c r="Y12">
         <v>8</v>
       </c>
-      <c r="V12">
+      <c r="Z12">
         <v>22</v>
       </c>
-      <c r="W12">
+      <c r="AA12">
         <v>58</v>
       </c>
-      <c r="X12">
+      <c r="AB12">
         <v>39</v>
       </c>
-      <c r="Y12">
+      <c r="AC12">
         <v>32</v>
       </c>
-      <c r="Z12">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+      <c r="AD12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>11</v>
       </c>
       <c r="B13">
+        <v>100</v>
+      </c>
+      <c r="C13">
+        <v>90</v>
+      </c>
+      <c r="D13">
+        <v>100</v>
+      </c>
+      <c r="E13">
+        <v>30</v>
+      </c>
+      <c r="F13">
         <v>40</v>
       </c>
-      <c r="C13">
+      <c r="G13">
         <v>65</v>
       </c>
-      <c r="D13">
-        <v>100</v>
-      </c>
-      <c r="E13">
+      <c r="H13">
+        <v>100</v>
+      </c>
+      <c r="I13">
         <v>88</v>
       </c>
-      <c r="F13">
-        <v>100</v>
-      </c>
-      <c r="G13">
-        <v>75</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
       <c r="J13">
+        <v>100</v>
+      </c>
+      <c r="K13">
+        <v>75</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
         <v>62</v>
       </c>
-      <c r="K13">
+      <c r="O13">
         <v>50</v>
       </c>
-      <c r="L13">
-        <v>100</v>
-      </c>
-      <c r="M13">
-        <v>100</v>
-      </c>
-      <c r="N13">
+      <c r="P13">
+        <v>100</v>
+      </c>
+      <c r="Q13">
+        <v>100</v>
+      </c>
+      <c r="R13">
         <v>77</v>
       </c>
-      <c r="O13">
-        <v>100</v>
-      </c>
-      <c r="P13">
+      <c r="S13">
+        <v>100</v>
+      </c>
+      <c r="T13">
         <v>65</v>
       </c>
-      <c r="Q13">
-        <v>100</v>
-      </c>
-      <c r="R13">
-        <v>100</v>
-      </c>
-      <c r="S13">
-        <v>100</v>
-      </c>
-      <c r="T13">
-        <v>100</v>
-      </c>
       <c r="U13">
         <v>100</v>
       </c>
@@ -1949,32 +2100,32 @@
         <v>100</v>
       </c>
       <c r="AC13">
+        <v>100</v>
+      </c>
+      <c r="AD13">
+        <v>100</v>
+      </c>
+      <c r="AE13">
+        <v>100</v>
+      </c>
+      <c r="AF13">
+        <v>100</v>
+      </c>
+      <c r="AG13">
         <v>80</v>
       </c>
-      <c r="AD13">
-        <v>100</v>
-      </c>
-      <c r="AE13">
+      <c r="AH13">
+        <v>100</v>
+      </c>
+      <c r="AI13">
         <v>83</v>
       </c>
-      <c r="AF13">
-        <v>100</v>
-      </c>
-      <c r="AG13">
+      <c r="AJ13">
+        <v>100</v>
+      </c>
+      <c r="AK13">
         <v>68</v>
       </c>
-      <c r="AH13">
-        <v>100</v>
-      </c>
-      <c r="AI13">
-        <v>100</v>
-      </c>
-      <c r="AJ13">
-        <v>100</v>
-      </c>
-      <c r="AK13">
-        <v>100</v>
-      </c>
       <c r="AL13">
         <v>100</v>
       </c>
@@ -2000,10 +2151,22 @@
         <v>100</v>
       </c>
       <c r="AT13">
+        <v>100</v>
+      </c>
+      <c r="AU13">
+        <v>100</v>
+      </c>
+      <c r="AV13">
+        <v>100</v>
+      </c>
+      <c r="AW13">
+        <v>100</v>
+      </c>
+      <c r="AX13">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -2014,106 +2177,106 @@
         <v>0</v>
       </c>
       <c r="D14">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>100</v>
+      </c>
+      <c r="I14">
         <v>130000</v>
       </c>
-      <c r="F14">
-        <v>100</v>
-      </c>
-      <c r="G14">
+      <c r="J14">
+        <v>100</v>
+      </c>
+      <c r="K14">
         <v>185000</v>
       </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
-      <c r="J14">
-        <v>0</v>
-      </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
       <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
         <v>20</v>
       </c>
-      <c r="M14">
+      <c r="Q14">
         <v>15</v>
       </c>
-      <c r="N14">
+      <c r="R14">
         <v>18</v>
       </c>
-      <c r="O14">
+      <c r="S14">
         <v>40</v>
       </c>
-      <c r="P14">
-        <v>0</v>
-      </c>
-      <c r="Q14">
-        <v>100</v>
-      </c>
-      <c r="R14">
-        <v>100</v>
-      </c>
-      <c r="S14">
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>100</v>
+      </c>
+      <c r="V14">
+        <v>100</v>
+      </c>
+      <c r="W14">
         <v>8</v>
       </c>
-      <c r="T14">
+      <c r="X14">
         <v>5</v>
       </c>
-      <c r="U14">
+      <c r="Y14">
         <v>8</v>
       </c>
-      <c r="V14">
+      <c r="Z14">
         <v>5</v>
       </c>
-      <c r="W14">
+      <c r="AA14">
         <v>17</v>
       </c>
-      <c r="X14">
+      <c r="AB14">
         <v>20</v>
       </c>
-      <c r="Y14">
+      <c r="AC14">
         <v>10</v>
       </c>
-      <c r="Z14">
+      <c r="AD14">
         <v>60</v>
       </c>
-      <c r="AA14">
+      <c r="AE14">
         <v>58</v>
       </c>
-      <c r="AB14">
-        <v>100</v>
-      </c>
-      <c r="AC14">
-        <v>0</v>
-      </c>
-      <c r="AD14">
+      <c r="AF14">
+        <v>100</v>
+      </c>
+      <c r="AG14">
+        <v>0</v>
+      </c>
+      <c r="AH14">
         <v>90</v>
       </c>
-      <c r="AE14">
-        <v>0</v>
-      </c>
-      <c r="AF14">
-        <v>0</v>
-      </c>
-      <c r="AG14">
-        <v>0</v>
-      </c>
-      <c r="AH14">
-        <v>100</v>
-      </c>
       <c r="AI14">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AJ14">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AK14">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AL14">
         <v>100</v>
@@ -2140,10 +2303,22 @@
         <v>100</v>
       </c>
       <c r="AT14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.55000000000000004">
+        <v>100</v>
+      </c>
+      <c r="AU14">
+        <v>100</v>
+      </c>
+      <c r="AV14">
+        <v>100</v>
+      </c>
+      <c r="AW14">
+        <v>100</v>
+      </c>
+      <c r="AX14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:50" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>62</v>
       </c>
@@ -2280,6 +2455,18 @@
         <v>100</v>
       </c>
       <c r="AT15">
+        <v>100</v>
+      </c>
+      <c r="AU15">
+        <v>100</v>
+      </c>
+      <c r="AV15">
+        <v>100</v>
+      </c>
+      <c r="AW15">
+        <v>100</v>
+      </c>
+      <c r="AX15">
         <v>100</v>
       </c>
     </row>
@@ -2291,17 +2478,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F45"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="50.578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.83984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.578125" customWidth="1"/>
-    <col min="5" max="5" width="10.578125" customWidth="1"/>
+    <col min="1" max="1" width="50.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.84375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="10.53515625" customWidth="1"/>
     <col min="6" max="6" width="48" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -2318,7 +2505,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2332,7 +2519,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -2346,7 +2533,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -2360,7 +2547,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -2371,7 +2558,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -2382,7 +2569,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -2393,7 +2580,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -2410,7 +2597,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>44</v>
       </c>
@@ -2427,7 +2614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>44</v>
       </c>
@@ -2444,7 +2631,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -2461,7 +2648,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -2478,7 +2665,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>44</v>
       </c>
@@ -2495,7 +2682,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -2509,7 +2696,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>56</v>
       </c>
@@ -2520,7 +2707,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -2534,7 +2721,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -2548,7 +2735,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -2565,7 +2752,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -2582,7 +2769,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2599,7 +2786,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -2616,7 +2803,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2633,7 +2820,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -2647,7 +2834,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -2664,7 +2851,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -2681,7 +2868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -2698,7 +2885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -2715,7 +2902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -2732,7 +2919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -2749,7 +2936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -2763,7 +2950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -2780,7 +2967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -2794,7 +2981,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -2808,7 +2995,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -2825,7 +3012,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>27</v>
       </c>
@@ -2842,7 +3029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>27</v>
       </c>
@@ -2859,7 +3046,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>27</v>
       </c>
@@ -2876,7 +3063,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -2893,7 +3080,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>27</v>
       </c>
@@ -2910,7 +3097,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -2927,7 +3114,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>27</v>
       </c>
@@ -2944,7 +3131,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>27</v>
       </c>
@@ -2961,7 +3148,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>27</v>
       </c>
@@ -2978,7 +3165,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>30</v>
       </c>
@@ -2992,7 +3179,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>30</v>
       </c>

</xml_diff>